<commit_message>
removed unrequired additional code
</commit_message>
<xml_diff>
--- a/ip_app.xlsx
+++ b/ip_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://curtin-my.sharepoint.com/personal/292636h_curtin_edu_au/Documents/PhD/Matlab/control-algorithm-ventilation/app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{B700CE7F-3E6B-4BDE-B908-FDFE437F02BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{328EB80F-D3B5-4E7E-9E33-0B89BABF65D5}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{B700CE7F-3E6B-4BDE-B908-FDFE437F02BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{126C0E27-699C-4B42-BCC7-9FB2F73DEEE8}"/>
   <bookViews>
-    <workbookView xWindow="28590" yWindow="4155" windowWidth="18900" windowHeight="10995" xr2:uid="{9F40D50C-DCAD-4A92-9C68-06D3A2E998A0}"/>
+    <workbookView xWindow="28245" yWindow="3810" windowWidth="18900" windowHeight="10995" xr2:uid="{9F40D50C-DCAD-4A92-9C68-06D3A2E998A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>pat</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>Q_cycle</t>
+  </si>
+  <si>
+    <t>triangle_paw</t>
   </si>
 </sst>
 </file>
@@ -484,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60D9B766-5E07-4599-8067-121ADA9FF2EF}">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -492,7 +495,7 @@
     <col min="17" max="17" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -533,10 +536,13 @@
         <v>23</v>
       </c>
       <c r="N1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -576,11 +582,14 @@
       <c r="M2">
         <v>0.3</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2">
+        <v>-1</v>
+      </c>
+      <c r="O2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -620,11 +629,14 @@
       <c r="M3">
         <v>0.3</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3">
+        <v>-1</v>
+      </c>
+      <c r="O3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -664,11 +676,14 @@
       <c r="M4">
         <v>0.3</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4">
+        <v>-1</v>
+      </c>
+      <c r="O4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -708,11 +723,14 @@
       <c r="M5">
         <v>0.3</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5">
+        <v>-1</v>
+      </c>
+      <c r="O5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -752,11 +770,14 @@
       <c r="M6">
         <v>0.3</v>
       </c>
-      <c r="N6" t="s">
+      <c r="N6">
+        <v>-1</v>
+      </c>
+      <c r="O6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -796,11 +817,14 @@
       <c r="M7">
         <v>0.3</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N7">
+        <v>-1</v>
+      </c>
+      <c r="O7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -840,11 +864,14 @@
       <c r="M8">
         <v>0.3</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N8">
+        <v>-1</v>
+      </c>
+      <c r="O8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -884,11 +911,14 @@
       <c r="M9">
         <v>0.3</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9">
+        <v>-1</v>
+      </c>
+      <c r="O9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -928,11 +958,14 @@
       <c r="M10">
         <v>0.3</v>
       </c>
-      <c r="N10" t="s">
+      <c r="N10">
+        <v>-1</v>
+      </c>
+      <c r="O10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -972,7 +1005,10 @@
       <c r="M11">
         <v>0.3</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N11">
+        <v>-1</v>
+      </c>
+      <c r="O11" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update ip files and account for T_onset
</commit_message>
<xml_diff>
--- a/ip_app.xlsx
+++ b/ip_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://curtin-my.sharepoint.com/personal/292636h_curtin_edu_au/Documents/PhD/Matlab/control-algorithm-ventilation/app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{B700CE7F-3E6B-4BDE-B908-FDFE437F02BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{126C0E27-699C-4B42-BCC7-9FB2F73DEEE8}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="8_{B700CE7F-3E6B-4BDE-B908-FDFE437F02BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0985D7E8-3F6F-423E-9001-BECE4DF708A9}"/>
   <bookViews>
-    <workbookView xWindow="28245" yWindow="3810" windowWidth="18900" windowHeight="10995" xr2:uid="{9F40D50C-DCAD-4A92-9C68-06D3A2E998A0}"/>
+    <workbookView xWindow="25080" yWindow="75" windowWidth="25440" windowHeight="15270" xr2:uid="{9F40D50C-DCAD-4A92-9C68-06D3A2E998A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>pat</t>
   </si>
@@ -77,40 +77,43 @@
     <t>file_general_model</t>
   </si>
   <si>
-    <t>pat_2_1004_0553_2110.mat</t>
-  </si>
-  <si>
-    <t>pat_4_2105_1606_1710_2210.mat</t>
-  </si>
-  <si>
-    <t>pat_5_1607_1930_2210_inv_resp_mech.mat</t>
-  </si>
-  <si>
-    <t>pat_6_1907_2330_2210_inv_resp_mech.mat</t>
-  </si>
-  <si>
-    <t>pat_7_2407_1118_2210.mat</t>
-  </si>
-  <si>
-    <t>pat_12_1611_1136_2210.mat</t>
-  </si>
-  <si>
-    <t>pat_17_2905_1855_2210.mat</t>
-  </si>
-  <si>
-    <t>pat_19_1706_1950_2210.mat</t>
-  </si>
-  <si>
-    <t>pat_22_0108_1030_2210.mat</t>
-  </si>
-  <si>
-    <t>pat_26_1802_1030_2210.mat</t>
-  </si>
-  <si>
     <t>Q_cycle</t>
   </si>
   <si>
     <t>triangle_paw</t>
+  </si>
+  <si>
+    <t>pat_1_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_2_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_3_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_4_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_5_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_6_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_7_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_8_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_9_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>pat_10_pmus_model.mat</t>
+  </si>
+  <si>
+    <t>T_onset</t>
   </si>
 </sst>
 </file>
@@ -487,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60D9B766-5E07-4599-8067-121ADA9FF2EF}">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -495,7 +498,7 @@
     <col min="17" max="17" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -533,16 +536,19 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="N1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="O1" t="s">
         <v>12</v>
       </c>
+      <c r="P1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -586,10 +592,13 @@
         <v>-1</v>
       </c>
       <c r="O2" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="P2">
+        <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -633,10 +642,13 @@
         <v>-1</v>
       </c>
       <c r="O3" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="P3">
+        <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -680,10 +692,13 @@
         <v>-1</v>
       </c>
       <c r="O4" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="P4">
+        <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -727,10 +742,13 @@
         <v>-1</v>
       </c>
       <c r="O5" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="P5">
+        <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -774,10 +792,13 @@
         <v>-1</v>
       </c>
       <c r="O6" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="P6">
+        <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -821,10 +842,13 @@
         <v>-1</v>
       </c>
       <c r="O7" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="P7">
+        <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -868,10 +892,13 @@
         <v>-1</v>
       </c>
       <c r="O8" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="P8">
+        <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -915,10 +942,13 @@
         <v>-1</v>
       </c>
       <c r="O9" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="P9">
+        <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -962,10 +992,13 @@
         <v>-1</v>
       </c>
       <c r="O10" t="s">
-        <v>21</v>
+        <v>23</v>
+      </c>
+      <c r="P10">
+        <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1009,7 +1042,10 @@
         <v>-1</v>
       </c>
       <c r="O11" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="P11">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>